<commit_message>
revision de los templates
</commit_message>
<xml_diff>
--- a/backend/templates/resumenFinal_template_.xlsx
+++ b/backend/templates/resumenFinal_template_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JavierWorkSpace\BatallaProject\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F45B74-786C-4502-BC26-9805BECFBB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE0904EB-9AB5-4F65-909F-1B403ADACB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="915" windowWidth="29040" windowHeight="15720" xr2:uid="{299BAFB4-AE58-4015-B36E-D7CD92F1B4DD}"/>
   </bookViews>
@@ -40,16 +40,292 @@
     <definedName name="inst_phone">'1er Año'!$U$8</definedName>
     <definedName name="inst_state">'1er Año'!$G$9</definedName>
     <definedName name="std_bd_1">'1er Año'!$K$16</definedName>
+    <definedName name="std_bd_10">'1er Año'!$K$25</definedName>
+    <definedName name="std_bd_11">'1er Año'!$K$26</definedName>
+    <definedName name="std_bd_12">'1er Año'!$K$27</definedName>
+    <definedName name="std_bd_13">'1er Año'!$K$28</definedName>
+    <definedName name="std_bd_14">'1er Año'!$K$29</definedName>
+    <definedName name="std_bd_15">'1er Año'!$K$30</definedName>
+    <definedName name="std_bd_16">'1er Año'!$K$31</definedName>
+    <definedName name="std_bd_17">'1er Año'!$K$32</definedName>
+    <definedName name="std_bd_18">'1er Año'!$K$33</definedName>
+    <definedName name="std_bd_19">'1er Año'!$K$34</definedName>
+    <definedName name="std_bd_2">'1er Año'!$K$17</definedName>
+    <definedName name="std_bd_20">'1er Año'!$K$35</definedName>
+    <definedName name="std_bd_21">'1er Año'!$K$36</definedName>
+    <definedName name="std_bd_22">'1er Año'!$K$37</definedName>
+    <definedName name="std_bd_23">'1er Año'!$K$38</definedName>
+    <definedName name="std_bd_24">'1er Año'!$K$39</definedName>
+    <definedName name="std_bd_25">'1er Año'!$K$40</definedName>
+    <definedName name="std_bd_26">'1er Año'!$K$41</definedName>
+    <definedName name="std_bd_27">'1er Año'!$K$42</definedName>
+    <definedName name="std_bd_28">'1er Año'!$K$43</definedName>
+    <definedName name="std_bd_29">'1er Año'!$K$44</definedName>
+    <definedName name="std_bd_3">'1er Año'!$K$18</definedName>
+    <definedName name="std_bd_30">'1er Año'!$K$45</definedName>
+    <definedName name="std_bd_31">'1er Año'!$K$46</definedName>
+    <definedName name="std_bd_32">'1er Año'!$K$47</definedName>
+    <definedName name="std_bd_33">'1er Año'!$K$48</definedName>
+    <definedName name="std_bd_34">'1er Año'!$K$49</definedName>
+    <definedName name="std_bd_35">'1er Año'!$K$50</definedName>
+    <definedName name="std_bd_4">'1er Año'!$K$19</definedName>
+    <definedName name="std_bd_5">'1er Año'!$K$20</definedName>
+    <definedName name="std_bd_6">'1er Año'!$K$21</definedName>
+    <definedName name="std_bd_7">'1er Año'!$K$22</definedName>
+    <definedName name="std_bd_8">'1er Año'!$K$23</definedName>
+    <definedName name="std_bd_9">'1er Año'!$K$24</definedName>
     <definedName name="std_bm_1">'1er Año'!$L$16</definedName>
+    <definedName name="std_bm_10">'1er Año'!$L$25</definedName>
+    <definedName name="std_bm_11">'1er Año'!$L$26</definedName>
+    <definedName name="std_bm_12">'1er Año'!$L$27</definedName>
+    <definedName name="std_bm_13">'1er Año'!$L$28</definedName>
+    <definedName name="std_bm_14">'1er Año'!$L$29</definedName>
+    <definedName name="std_bm_15">'1er Año'!$L$30</definedName>
+    <definedName name="std_bm_16">'1er Año'!$L$31</definedName>
+    <definedName name="std_bm_17">'1er Año'!$L$32</definedName>
+    <definedName name="std_bm_18">'1er Año'!$L$33</definedName>
+    <definedName name="std_bm_19">'1er Año'!$L$34</definedName>
+    <definedName name="std_bm_2">'1er Año'!$L$17</definedName>
+    <definedName name="std_bm_20">'1er Año'!$L$35</definedName>
+    <definedName name="std_bm_21">'1er Año'!$L$36</definedName>
+    <definedName name="std_bm_22">'1er Año'!$L$37</definedName>
+    <definedName name="std_bm_23">'1er Año'!$L$38</definedName>
+    <definedName name="std_bm_24">'1er Año'!$L$39</definedName>
+    <definedName name="std_bm_25">'1er Año'!$L$40</definedName>
+    <definedName name="std_bm_26">'1er Año'!$L$41</definedName>
+    <definedName name="std_bm_27">'1er Año'!$L$42</definedName>
+    <definedName name="std_bm_28">'1er Año'!$L$43</definedName>
+    <definedName name="std_bm_29">'1er Año'!$L$44</definedName>
+    <definedName name="std_bm_3">'1er Año'!$L$18</definedName>
+    <definedName name="std_bm_30">'1er Año'!$L$45</definedName>
+    <definedName name="std_bm_31">'1er Año'!$L$46</definedName>
+    <definedName name="std_bm_32">'1er Año'!$L$47</definedName>
+    <definedName name="std_bm_33">'1er Año'!$L$48</definedName>
+    <definedName name="std_bm_34">'1er Año'!$L$49</definedName>
+    <definedName name="std_bm_35">'1er Año'!$L$50</definedName>
+    <definedName name="std_bm_4">'1er Año'!$L$19</definedName>
+    <definedName name="std_bm_5">'1er Año'!$L$20</definedName>
+    <definedName name="std_bm_6">'1er Año'!$L$21</definedName>
+    <definedName name="std_bm_7">'1er Año'!$L$22</definedName>
+    <definedName name="std_bm_8">'1er Año'!$L$23</definedName>
+    <definedName name="std_bm_9">'1er Año'!$L$24</definedName>
     <definedName name="std_bp_1">'1er Año'!$H$16</definedName>
+    <definedName name="std_bp_10">'1er Año'!$H$25</definedName>
+    <definedName name="std_bp_11">'1er Año'!$H$26</definedName>
+    <definedName name="std_bp_12">'1er Año'!$H$27</definedName>
+    <definedName name="std_bp_13">'1er Año'!$H$28</definedName>
+    <definedName name="std_bp_14">'1er Año'!$H$29</definedName>
+    <definedName name="std_bp_15">'1er Año'!$H$30</definedName>
+    <definedName name="std_bp_16">'1er Año'!$H$31</definedName>
+    <definedName name="std_bp_17">'1er Año'!$H$32</definedName>
+    <definedName name="std_bp_18">'1er Año'!$H$33</definedName>
+    <definedName name="std_bp_19">'1er Año'!$H$34</definedName>
+    <definedName name="std_bp_2">'1er Año'!$H$17</definedName>
+    <definedName name="std_bp_20">'1er Año'!$H$35</definedName>
+    <definedName name="std_bp_21">'1er Año'!$H$36</definedName>
+    <definedName name="std_bp_22">'1er Año'!$H$37</definedName>
+    <definedName name="std_bp_23">'1er Año'!$H$38</definedName>
+    <definedName name="std_bp_24">'1er Año'!$H$39</definedName>
+    <definedName name="std_bp_25">'1er Año'!$H$40</definedName>
+    <definedName name="std_bp_26">'1er Año'!$H$41</definedName>
+    <definedName name="std_bp_27">'1er Año'!$H$42</definedName>
+    <definedName name="std_bp_28">'1er Año'!$H$43</definedName>
+    <definedName name="std_bp_29">'1er Año'!$H$44</definedName>
+    <definedName name="std_bp_3">'1er Año'!$H$18</definedName>
+    <definedName name="std_bp_30">'1er Año'!$H$45</definedName>
+    <definedName name="std_bp_31">'1er Año'!$H$46</definedName>
+    <definedName name="std_bp_32">'1er Año'!$H$47</definedName>
+    <definedName name="std_bp_33">'1er Año'!$H$48</definedName>
+    <definedName name="std_bp_34">'1er Año'!$H$49</definedName>
+    <definedName name="std_bp_35">'1er Año'!$H$50</definedName>
+    <definedName name="std_bp_4">'1er Año'!$H$19</definedName>
+    <definedName name="std_bp_5">'1er Año'!$H$20</definedName>
+    <definedName name="std_bp_6">'1er Año'!$H$21</definedName>
+    <definedName name="std_bp_7">'1er Año'!$H$22</definedName>
+    <definedName name="std_bp_8">'1er Año'!$H$23</definedName>
+    <definedName name="std_bp_9">'1er Año'!$H$24</definedName>
     <definedName name="std_by_1">'1er Año'!$M$16</definedName>
+    <definedName name="std_by_2">'1er Año'!$M$17</definedName>
+    <definedName name="std_by_3">'1er Año'!$M$18</definedName>
+    <definedName name="std_by_4">'1er Año'!$M$19</definedName>
+    <definedName name="std_by_5">'1er Año'!$M$20</definedName>
     <definedName name="std_doc_1">'1er Año'!$B$16</definedName>
+    <definedName name="std_doc_10">'1er Año'!$B$25</definedName>
+    <definedName name="std_doc_11">'1er Año'!$B$26</definedName>
+    <definedName name="std_doc_12">'1er Año'!$B$27</definedName>
+    <definedName name="std_doc_13">'1er Año'!$B$28</definedName>
+    <definedName name="std_doc_14">'1er Año'!$B$29</definedName>
+    <definedName name="std_doc_15">'1er Año'!$B$30</definedName>
+    <definedName name="std_doc_16">'1er Año'!$B$31</definedName>
+    <definedName name="std_doc_17">'1er Año'!$B$32</definedName>
+    <definedName name="std_doc_18">'1er Año'!$B$33</definedName>
+    <definedName name="std_doc_19">'1er Año'!$B$34</definedName>
+    <definedName name="std_doc_2">'1er Año'!$B$17</definedName>
+    <definedName name="std_doc_20">'1er Año'!$B$35</definedName>
+    <definedName name="std_doc_21">'1er Año'!$B$36</definedName>
+    <definedName name="std_doc_22">'1er Año'!$B$37</definedName>
+    <definedName name="std_doc_23">'1er Año'!$B$38</definedName>
+    <definedName name="std_doc_24">'1er Año'!$B$39</definedName>
+    <definedName name="std_doc_25">'1er Año'!$B$40</definedName>
+    <definedName name="std_doc_26">'1er Año'!$B$41</definedName>
+    <definedName name="std_doc_27">'1er Año'!$B$42</definedName>
+    <definedName name="std_doc_28">'1er Año'!$B$43</definedName>
+    <definedName name="std_doc_29">'1er Año'!$B$44</definedName>
+    <definedName name="std_doc_3">'1er Año'!$B$18</definedName>
+    <definedName name="std_doc_30">'1er Año'!$B$45</definedName>
+    <definedName name="std_doc_31">'1er Año'!$B$46</definedName>
+    <definedName name="std_doc_32">'1er Año'!$B$47</definedName>
+    <definedName name="std_doc_33">'1er Año'!$B$48</definedName>
+    <definedName name="std_doc_34">'1er Año'!$B$49</definedName>
+    <definedName name="std_doc_35">'1er Año'!$B$50</definedName>
+    <definedName name="std_doc_4">'1er Año'!$B$19</definedName>
+    <definedName name="std_doc_5">'1er Año'!$B$20</definedName>
+    <definedName name="std_doc_6">'1er Año'!$B$21</definedName>
+    <definedName name="std_doc_7">'1er Año'!$B$22</definedName>
+    <definedName name="std_doc_8">'1er Año'!$B$23</definedName>
+    <definedName name="std_doc_9">'1er Año'!$B$24</definedName>
     <definedName name="std_ef_1">'1er Año'!$I$16</definedName>
+    <definedName name="std_ef_10">'1er Año'!$I$25</definedName>
+    <definedName name="std_ef_11">'1er Año'!$I$26</definedName>
+    <definedName name="std_ef_12">'1er Año'!$I$27</definedName>
+    <definedName name="std_ef_13">'1er Año'!$I$28</definedName>
+    <definedName name="std_ef_14">'1er Año'!$I$29</definedName>
+    <definedName name="std_ef_15">'1er Año'!$I$30</definedName>
+    <definedName name="std_ef_16">'1er Año'!$I$31</definedName>
+    <definedName name="std_ef_17">'1er Año'!$I$32</definedName>
+    <definedName name="std_ef_18">'1er Año'!$I$33</definedName>
+    <definedName name="std_ef_19">'1er Año'!$I$34</definedName>
+    <definedName name="std_ef_2">'1er Año'!$I$17</definedName>
+    <definedName name="std_ef_20">'1er Año'!$I$35</definedName>
+    <definedName name="std_ef_21">'1er Año'!$I$36</definedName>
+    <definedName name="std_ef_22">'1er Año'!$I$37</definedName>
+    <definedName name="std_ef_23">'1er Año'!$I$38</definedName>
+    <definedName name="std_ef_24">'1er Año'!$I$39</definedName>
+    <definedName name="std_ef_25">'1er Año'!$I$40</definedName>
+    <definedName name="std_ef_26">'1er Año'!$I$41</definedName>
+    <definedName name="std_ef_27">'1er Año'!$I$42</definedName>
+    <definedName name="std_ef_28">'1er Año'!$I$43</definedName>
+    <definedName name="std_ef_29">'1er Año'!$I$44</definedName>
+    <definedName name="std_ef_3">'1er Año'!$I$18</definedName>
+    <definedName name="std_ef_30">'1er Año'!$I$45</definedName>
+    <definedName name="std_ef_31">'1er Año'!$I$46</definedName>
+    <definedName name="std_ef_32">'1er Año'!$I$47</definedName>
+    <definedName name="std_ef_33">'1er Año'!$I$48</definedName>
+    <definedName name="std_ef_34">'1er Año'!$I$49</definedName>
+    <definedName name="std_ef_35">'1er Año'!$I$50</definedName>
+    <definedName name="std_ef_4">'1er Año'!$I$19</definedName>
+    <definedName name="std_ef_5">'1er Año'!$I$20</definedName>
+    <definedName name="std_ef_6">'1er Año'!$I$21</definedName>
+    <definedName name="std_ef_7">'1er Año'!$I$22</definedName>
+    <definedName name="std_ef_8">'1er Año'!$I$23</definedName>
+    <definedName name="std_ef_9">'1er Año'!$I$24</definedName>
     <definedName name="std_fn_1">'1er Año'!$F$16</definedName>
+    <definedName name="std_fn_10">'1er Año'!$F$25</definedName>
+    <definedName name="std_fn_11">'1er Año'!$F$26</definedName>
+    <definedName name="std_fn_12">'1er Año'!$F$27</definedName>
+    <definedName name="std_fn_13">'1er Año'!$F$28</definedName>
+    <definedName name="std_fn_14">'1er Año'!$F$29</definedName>
+    <definedName name="std_fn_15">'1er Año'!$F$30</definedName>
+    <definedName name="std_fn_16">'1er Año'!$F$31</definedName>
+    <definedName name="std_fn_17">'1er Año'!$F$32</definedName>
+    <definedName name="std_fn_18">'1er Año'!$F$33</definedName>
+    <definedName name="std_fn_19">'1er Año'!$F$34</definedName>
+    <definedName name="std_fn_2">'1er Año'!$F$17</definedName>
+    <definedName name="std_fn_20">'1er Año'!$F$35</definedName>
+    <definedName name="std_fn_21">'1er Año'!$F$36</definedName>
+    <definedName name="std_fn_22">'1er Año'!$F$37</definedName>
+    <definedName name="std_fn_23">'1er Año'!$F$38</definedName>
+    <definedName name="std_fn_24">'1er Año'!$F$39</definedName>
+    <definedName name="std_fn_25">'1er Año'!$F$40</definedName>
+    <definedName name="std_fn_26">'1er Año'!$F$41</definedName>
+    <definedName name="std_fn_27">'1er Año'!$F$42</definedName>
+    <definedName name="std_fn_28">'1er Año'!$F$43</definedName>
+    <definedName name="std_fn_29">'1er Año'!$F$44</definedName>
+    <definedName name="std_fn_3">'1er Año'!$F$18</definedName>
+    <definedName name="std_fn_30">'1er Año'!$F$45</definedName>
+    <definedName name="std_fn_31">'1er Año'!$F$46</definedName>
+    <definedName name="std_fn_32">'1er Año'!$F$47</definedName>
+    <definedName name="std_fn_33">'1er Año'!$F$48</definedName>
+    <definedName name="std_fn_34">'1er Año'!$F$49</definedName>
+    <definedName name="std_fn_35">'1er Año'!$F$50</definedName>
+    <definedName name="std_fn_4">'1er Año'!$F$19</definedName>
+    <definedName name="std_fn_5">'1er Año'!$F$20</definedName>
+    <definedName name="std_fn_6">'1er Año'!$F$21</definedName>
+    <definedName name="std_fn_7">'1er Año'!$F$22</definedName>
+    <definedName name="std_fn_8">'1er Año'!$F$23</definedName>
+    <definedName name="std_fn_9">'1er Año'!$F$24</definedName>
     <definedName name="std_ln_1">'1er Año'!$D$16</definedName>
+    <definedName name="std_ln_10">'1er Año'!$D$25</definedName>
+    <definedName name="std_ln_11">'1er Año'!$D$26</definedName>
+    <definedName name="std_ln_12">'1er Año'!$D$27</definedName>
+    <definedName name="std_ln_13">'1er Año'!$D$28</definedName>
+    <definedName name="std_ln_14">'1er Año'!$D$29</definedName>
+    <definedName name="std_ln_15">'1er Año'!$D$30</definedName>
+    <definedName name="std_ln_16">'1er Año'!$D$31</definedName>
+    <definedName name="std_ln_17">'1er Año'!$D$32</definedName>
+    <definedName name="std_ln_18">'1er Año'!$D$33</definedName>
+    <definedName name="std_ln_19">'1er Año'!$D$34</definedName>
+    <definedName name="std_ln_2">'1er Año'!$D$17</definedName>
+    <definedName name="std_ln_20">'1er Año'!$D$35</definedName>
+    <definedName name="std_ln_21">'1er Año'!$D$36</definedName>
+    <definedName name="std_ln_22">'1er Año'!$D$37</definedName>
+    <definedName name="std_ln_23">'1er Año'!$D$38</definedName>
+    <definedName name="std_ln_24">'1er Año'!$D$39</definedName>
+    <definedName name="std_ln_25">'1er Año'!$D$40</definedName>
+    <definedName name="std_ln_26">'1er Año'!$D$41</definedName>
+    <definedName name="std_ln_27">'1er Año'!$D$42</definedName>
+    <definedName name="std_ln_28">'1er Año'!$D$43</definedName>
+    <definedName name="std_ln_29">'1er Año'!$D$44</definedName>
+    <definedName name="std_ln_3">'1er Año'!$D$18</definedName>
+    <definedName name="std_ln_30">'1er Año'!$D$45</definedName>
+    <definedName name="std_ln_31">'1er Año'!$D$46</definedName>
+    <definedName name="std_ln_32">'1er Año'!$D$47</definedName>
+    <definedName name="std_ln_33">'1er Año'!$D$48</definedName>
+    <definedName name="std_ln_34">'1er Año'!$D$49</definedName>
+    <definedName name="std_ln_35">'1er Año'!$D$50</definedName>
+    <definedName name="std_ln_4">'1er Año'!$D$19</definedName>
+    <definedName name="std_ln_5">'1er Año'!$D$20</definedName>
+    <definedName name="std_ln_6">'1er Año'!$D$21</definedName>
+    <definedName name="std_ln_7">'1er Año'!$D$22</definedName>
+    <definedName name="std_ln_8">'1er Año'!$D$23</definedName>
+    <definedName name="std_ln_9">'1er Año'!$D$24</definedName>
     <definedName name="std_ln_n">'1er Año'!$D$16</definedName>
     <definedName name="std_num_1">'1er Año'!$V$15</definedName>
     <definedName name="std_sx_1">'1er Año'!$J$16</definedName>
+    <definedName name="std_sx_10">'1er Año'!$J$25</definedName>
+    <definedName name="std_sx_11">'1er Año'!$J$26</definedName>
+    <definedName name="std_sx_12">'1er Año'!$J$27</definedName>
+    <definedName name="std_sx_13">'1er Año'!$J$28</definedName>
+    <definedName name="std_sx_14">'1er Año'!$J$29</definedName>
+    <definedName name="std_sx_15">'1er Año'!$J$30</definedName>
+    <definedName name="std_sx_16">'1er Año'!$J$31</definedName>
+    <definedName name="std_sx_17">'1er Año'!$J$32</definedName>
+    <definedName name="std_sx_18">'1er Año'!$J$33</definedName>
+    <definedName name="std_sx_19">'1er Año'!$J$34</definedName>
+    <definedName name="std_sx_2">'1er Año'!$J$17</definedName>
+    <definedName name="std_sx_20">'1er Año'!$J$35</definedName>
+    <definedName name="std_sx_21">'1er Año'!$J$36</definedName>
+    <definedName name="std_sx_22">'1er Año'!$J$37</definedName>
+    <definedName name="std_sx_23">'1er Año'!$J$38</definedName>
+    <definedName name="std_sx_24">'1er Año'!$J$39</definedName>
+    <definedName name="std_sx_25">'1er Año'!$J$40</definedName>
+    <definedName name="std_sx_26">'1er Año'!$J$41</definedName>
+    <definedName name="std_sx_27">'1er Año'!$J$42</definedName>
+    <definedName name="std_sx_28">'1er Año'!$J$43</definedName>
+    <definedName name="std_sx_29">'1er Año'!$J$44</definedName>
+    <definedName name="std_sx_3">'1er Año'!$J$18</definedName>
+    <definedName name="std_sx_30">'1er Año'!$J$45</definedName>
+    <definedName name="std_sx_31">'1er Año'!$J$46</definedName>
+    <definedName name="std_sx_32">'1er Año'!$J$47</definedName>
+    <definedName name="std_sx_33">'1er Año'!$J$48</definedName>
+    <definedName name="std_sx_34">'1er Año'!$J$49</definedName>
+    <definedName name="std_sx_35">'1er Año'!$J$50</definedName>
+    <definedName name="std_sx_4">'1er Año'!$J$19</definedName>
+    <definedName name="std_sx_5">'1er Año'!$J$20</definedName>
+    <definedName name="std_sx_6">'1er Año'!$J$21</definedName>
+    <definedName name="std_sx_7">'1er Año'!$J$22</definedName>
+    <definedName name="std_sx_8">'1er Año'!$J$23</definedName>
+    <definedName name="std_sx_9">'1er Año'!$J$24</definedName>
     <definedName name="subj_1">'1er Año'!$N$15</definedName>
     <definedName name="subj_2">'1er Año'!$O$15</definedName>
     <definedName name="subj_3">'1er Año'!$P$15</definedName>
@@ -59,18 +335,39 @@
     <definedName name="subj_7">'1er Año'!$T$15</definedName>
     <definedName name="subj_8">'1er Año'!$U$15</definedName>
     <definedName name="subj_9">'1er Año'!$V$15</definedName>
+    <definedName name="subjname_1">'1er Año'!$C$58</definedName>
+    <definedName name="subjname_2">'1er Año'!$C$59</definedName>
+    <definedName name="subjname_3">'1er Año'!$C$60</definedName>
+    <definedName name="subjname_4">'1er Año'!$C$61</definedName>
+    <definedName name="subjname_5">'1er Año'!$C$62</definedName>
+    <definedName name="subjname_6">'1er Año'!$C$63</definedName>
+    <definedName name="subjname_7">'1er Año'!$C$64</definedName>
+    <definedName name="subjname_8">'1er Año'!$C$65</definedName>
+    <definedName name="subjname_9">'1er Año'!$C$66</definedName>
+    <definedName name="subjname_i7">'1er Año'!$C$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="153">
   <si>
     <t>Artes Gráficas</t>
   </si>
@@ -505,18 +802,6 @@
     <t>RESUMEN FINAL DEL RENDIMIENTO ESTUDIANTIL</t>
   </si>
   <si>
-    <t>AP</t>
-  </si>
-  <si>
-    <t>CN</t>
-  </si>
-  <si>
-    <t>Arte y Patrimonio</t>
-  </si>
-  <si>
-    <t>Ciencias Naturales</t>
-  </si>
-  <si>
     <t>PRIMERO</t>
   </si>
   <si>
@@ -539,6 +824,9 @@
   </si>
   <si>
     <t>*</t>
+  </si>
+  <si>
+    <t>****************************</t>
   </si>
 </sst>
 </file>
@@ -913,9 +1201,6 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -924,6 +1209,9 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1913,7 +2201,7 @@
       <c r="L4" s="133"/>
       <c r="M4" s="133"/>
       <c r="N4" s="135" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O4" s="135"/>
       <c r="P4" s="135"/>
@@ -2315,31 +2603,31 @@
       <c r="L15" s="122"/>
       <c r="M15" s="122"/>
       <c r="N15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="R15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="S15" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="T15" s="20" t="s">
-        <v>155</v>
+        <v>151</v>
+      </c>
+      <c r="T15" s="19" t="s">
+        <v>151</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="V15" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="W15" s="35"/>
       <c r="X15" s="36"/>
@@ -3660,11 +3948,12 @@
       <c r="A58" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B58" s="19" t="s">
-        <v>64</v>
+      <c r="B58" s="22" t="str">
+        <f>subj_1</f>
+        <v>*</v>
       </c>
       <c r="C58" s="77" t="s">
-        <v>82</v>
+        <v>152</v>
       </c>
       <c r="D58" s="78"/>
       <c r="E58" s="79"/>
@@ -3696,11 +3985,12 @@
       <c r="A59" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B59" s="19" t="s">
-        <v>65</v>
+      <c r="B59" s="22" t="str">
+        <f>subj_2</f>
+        <v>*</v>
       </c>
       <c r="C59" s="77" t="s">
-        <v>83</v>
+        <v>152</v>
       </c>
       <c r="D59" s="78"/>
       <c r="E59" s="79"/>
@@ -3732,11 +4022,12 @@
       <c r="A60" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B60" s="19" t="s">
-        <v>66</v>
+      <c r="B60" s="22" t="str">
+        <f>subj_3</f>
+        <v>*</v>
       </c>
       <c r="C60" s="77" t="s">
-        <v>84</v>
+        <v>152</v>
       </c>
       <c r="D60" s="78"/>
       <c r="E60" s="79"/>
@@ -3768,11 +4059,12 @@
       <c r="A61" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B61" s="19" t="s">
-        <v>44</v>
+      <c r="B61" s="22" t="str">
+        <f>subj_4</f>
+        <v>*</v>
       </c>
       <c r="C61" s="77" t="s">
-        <v>85</v>
+        <v>152</v>
       </c>
       <c r="D61" s="78"/>
       <c r="E61" s="79"/>
@@ -3804,11 +4096,12 @@
       <c r="A62" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B62" s="19" t="s">
-        <v>144</v>
+      <c r="B62" s="22" t="str">
+        <f>subj_5</f>
+        <v>*</v>
       </c>
       <c r="C62" s="77" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="D62" s="78"/>
       <c r="E62" s="79"/>
@@ -3823,7 +4116,7 @@
       <c r="N62" s="82"/>
       <c r="O62" s="81"/>
       <c r="P62" s="89" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="Q62" s="90"/>
       <c r="R62" s="90"/>
@@ -3840,11 +4133,12 @@
       <c r="A63" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B63" s="19" t="s">
-        <v>145</v>
+      <c r="B63" s="22" t="str">
+        <f>subj_6</f>
+        <v>*</v>
       </c>
       <c r="C63" s="77" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D63" s="78"/>
       <c r="E63" s="79"/>
@@ -3876,11 +4170,12 @@
       <c r="A64" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>71</v>
+      <c r="B64" s="22" t="str">
+        <f>subj_7</f>
+        <v>*</v>
       </c>
       <c r="C64" s="77" t="s">
-        <v>90</v>
+        <v>152</v>
       </c>
       <c r="D64" s="78"/>
       <c r="E64" s="79"/>
@@ -3912,11 +4207,12 @@
       <c r="A65" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B65" s="19" t="s">
-        <v>73</v>
+      <c r="B65" s="22" t="str">
+        <f>subj_8</f>
+        <v>*</v>
       </c>
       <c r="C65" s="77" t="s">
-        <v>92</v>
+        <v>152</v>
       </c>
       <c r="D65" s="78"/>
       <c r="E65" s="79"/>
@@ -3950,8 +4246,9 @@
       <c r="A66" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B66" s="21" t="s">
-        <v>154</v>
+      <c r="B66" s="22" t="str">
+        <f>subj_9</f>
+        <v>*</v>
       </c>
       <c r="C66" s="83" t="s">
         <v>123</v>
@@ -4642,7 +4939,7 @@
       <c r="L4" s="133"/>
       <c r="M4" s="133"/>
       <c r="N4" s="135" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O4" s="135"/>
       <c r="P4" s="135"/>
@@ -5066,14 +5363,14 @@
       <c r="T15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="U15" s="20" t="s">
+      <c r="U15" s="19" t="s">
         <v>71</v>
       </c>
       <c r="V15" s="3" t="s">
         <v>73</v>
       </c>
       <c r="W15" s="13" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="X15" s="35"/>
       <c r="Y15" s="36"/>
@@ -6558,7 +6855,7 @@
       <c r="N62" s="82"/>
       <c r="O62" s="81"/>
       <c r="P62" s="89" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="Q62" s="90"/>
       <c r="R62" s="90"/>
@@ -6719,8 +7016,8 @@
       <c r="A67" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B67" s="21" t="s">
-        <v>154</v>
+      <c r="B67" s="20" t="s">
+        <v>150</v>
       </c>
       <c r="C67" s="83" t="s">
         <v>123</v>
@@ -7414,7 +7711,7 @@
       <c r="L4" s="133"/>
       <c r="M4" s="133"/>
       <c r="N4" s="135" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O4" s="135"/>
       <c r="P4" s="135"/>
@@ -7840,17 +8137,17 @@
       <c r="T15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="U15" s="20" t="s">
+      <c r="U15" s="19" t="s">
         <v>71</v>
       </c>
       <c r="V15" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="W15" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="X15" s="22" t="s">
-        <v>153</v>
+      <c r="X15" s="21" t="s">
+        <v>149</v>
       </c>
       <c r="Y15" s="35"/>
       <c r="Z15" s="37"/>
@@ -9334,7 +9631,7 @@
       <c r="N62" s="82"/>
       <c r="O62" s="81"/>
       <c r="P62" s="89" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="Q62" s="90"/>
       <c r="R62" s="90"/>
@@ -9458,7 +9755,7 @@
         <v>9</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C66" s="77" t="s">
         <v>91</v>
@@ -9529,8 +9826,8 @@
       <c r="A68" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B68" s="21" t="s">
-        <v>154</v>
+      <c r="B68" s="20" t="s">
+        <v>150</v>
       </c>
       <c r="C68" s="83" t="s">
         <v>123</v>
@@ -10226,7 +10523,7 @@
       <c r="L4" s="133"/>
       <c r="M4" s="133"/>
       <c r="N4" s="131" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O4" s="131"/>
       <c r="P4" s="131"/>
@@ -10657,7 +10954,7 @@
       <c r="U15" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="V15" s="20" t="s">
+      <c r="V15" s="19" t="s">
         <v>71</v>
       </c>
       <c r="W15" s="3" t="s">
@@ -10666,8 +10963,8 @@
       <c r="X15" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="Y15" s="22" t="s">
-        <v>153</v>
+      <c r="Y15" s="21" t="s">
+        <v>149</v>
       </c>
       <c r="Z15" s="140"/>
     </row>
@@ -12318,7 +12615,7 @@
         <v>10</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C67" s="77" t="s">
         <v>91</v>
@@ -12389,8 +12686,8 @@
       <c r="A69" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="21" t="s">
-        <v>154</v>
+      <c r="B69" s="20" t="s">
+        <v>150</v>
       </c>
       <c r="C69" s="83" t="s">
         <v>123</v>

</xml_diff>